<commit_message>
regulation: 2026-10-26 (+3 новых, ~1 изменено, −0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/lab/regulation-en.xlsx
+++ b/public/lab/regulation-en.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Country summary'!$A$1:$M$21</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Rules!$A$1:$J$26</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Rules!$A$1:$J$29</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="281">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -457,42 +457,42 @@
     <t xml:space="preserve">https://vinciworks.com/blog/eudr-delayed-again-what-changed-what-is-now-fixed-and-what-businesses-should-do-in-2026/</t>
   </si>
   <si>
+    <t xml:space="preserve">30.12.2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delegated Regulation (EU) 2026/2102 of 13 Jul 2026 (OJ 17 Sep 2026), amending Annex I to EUDR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUDR extended to palm oil derivatives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adopted; in force since 18 Sep 2026. Adds oil-palm derivatives to the EUDR list: hydrogenated and chemically modified palm oils (ex 1516 20, ex 1518), crude glycerol, fatty alcohols, acids and esters, amines, soap (ex 3401), chemical preparations (ex 3824 99), polyethers. New entries apply from 30 Dec 2027.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://eur-lex.europa.eu/eli/reg_del/2026/2102/oj/eng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EAEU (common rules)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.07.2013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR CU 022/2011 “Food products: labelling”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generic ‘vegetable oil’ name allowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refined oils may be listed as ‘vegetable oil (fat)’ without the species — the main loophole for not naming palm oil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://eec.eaeunion.org/comission/department/deptexreg/tr/PischevkaMarkirovka.php</t>
+  </si>
+  <si>
     <t xml:space="preserve">Proposal / draft</t>
   </si>
   <si>
-    <t xml:space="preserve">04.05.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft delegated act under EUDR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EUDR extended to palm oil derivatives</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Commission proposed adding oleochemicals (fatty acids, their esters, palm-based soap).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://blog.foodsconnected.com/7-key-takeaways-from-the-april-2026-eudr-review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EAEU (common rules)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01.07.2013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR CU 022/2011 “Food products: labelling”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generic ‘vegetable oil’ name allowed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refined oils may be listed as ‘vegetable oil (fat)’ without the species — the main loophole for not naming palm oil.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://eec.eaeunion.org/comission/department/deptexreg/tr/PischevkaMarkirovka.php</t>
-  </si>
-  <si>
     <t xml:space="preserve">Amendments to TR CU 022/2011 (drafted by Belarus)</t>
   </si>
   <si>
@@ -523,6 +523,21 @@
     <t xml:space="preserve">https://foodsmi.com/zakonodatelstvo/izmeneniya-v-tekhreglamente-na-maslozhirovuyu-produktsiyu/</t>
   </si>
   <si>
+    <t xml:space="preserve">28.12.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EEC Board Decision No. 80 of 29 Jun 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New lists of standards for TR CU 024/2011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approves the list of standards whose voluntary use ensures compliance with TR CU 024/2011 on oil and fat products (50 items) and the list of test and sampling methods (183 items). Replaces EEC Board Decision No. 53 of 29 Mar 2022. Enters into force 180 days after publication — 28 Dec 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://base.spinform.ru/show_doc.fwx?rgn=177646</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dairy and milk fat substitutes</t>
   </si>
   <si>
@@ -601,6 +616,24 @@
     <t xml:space="preserve">https://www.retail.ru/news/v-rossii-poyavilsya-edinyy-katalog-produktov-bez-palmy-23-dekabrya-2025-272975/</t>
   </si>
   <si>
+    <t xml:space="preserve">Taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.10.2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal Law No. 268-FZ of 2 Aug 2019 (Art. 164 Tax Code); Government Decree No. 849 of 11 May 2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20% VAT on palm oil instead of reduced 10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palm oil removed from the list of foods with the reduced 10% VAT rate from 1 Oct 2019; from 1 Jul 2022 the 20% rate also applies to palm oil fractions (on import and sale).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.v2b.ru/documents/federalnyy-zakon-ot-02-08-2019-268-fz/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Digital marking and traceability</t>
   </si>
   <si>
@@ -664,6 +697,21 @@
     <t xml:space="preserve">https://ria.ru/20260722/markirovka-2106133235.html</t>
   </si>
   <si>
+    <t xml:space="preserve">22.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V. Volodin at the State Duma plenary, 22 Oct 2026; S. Mironov proposal, 24 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palm oil ban in baby food and in school/hospital procurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The State Duma speaker proposed discussing a ban on palm oil in children’s food and higher taxation of palm oil. The A Just Russia faction leader proposed a federal law banning medical and educational institutions from buying food containing palm oil. No bill has been introduced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ria.ru/20261024/maslo-2126771171.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">01.04.2027</t>
   </si>
   <si>
@@ -733,9 +781,6 @@
     <t xml:space="preserve">https://podrobno.uz/cat/obchestvo/v-uzbekistane-vvodyat-obyazatelnyy-laboratornyy-kontrol-palmovogo-masla-i-transzhirov/</t>
   </si>
   <si>
-    <t xml:space="preserve">Taxes</t>
-  </si>
-  <si>
     <t xml:space="preserve">30.07.2026</t>
   </si>
   <si>
@@ -793,7 +838,7 @@
     <t xml:space="preserve">Data as of</t>
   </si>
   <si>
-    <t xml:space="preserve">23.10.2026</t>
+    <t xml:space="preserve">26.10.2026</t>
   </si>
   <si>
     <t xml:space="preserve">Review period</t>
@@ -1441,20 +1486,20 @@
         <v>16</v>
       </c>
       <c r="F2" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L2)+COUNTIF(Rules!$B$2:$B$26,M2)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L2)+COUNTIF(Rules!$B$2:$B$29,M2)</f>
         <v>5</v>
       </c>
       <c r="G2" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L2,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M2,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L2,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M2,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H2" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L2,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M2,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L2,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M2,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I2" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L2,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M2,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L2,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M2,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>17</v>
@@ -1486,20 +1531,20 @@
         <v>16</v>
       </c>
       <c r="F3" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L3)+COUNTIF(Rules!$B$2:$B$26,M3)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L3)+COUNTIF(Rules!$B$2:$B$29,M3)</f>
         <v>5</v>
       </c>
       <c r="G3" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L3,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M3,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L3,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M3,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H3" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L3,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M3,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L3,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M3,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I3" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L3,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M3,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L3,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M3,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>17</v>
@@ -1531,20 +1576,20 @@
         <v>26</v>
       </c>
       <c r="F4" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L4)+COUNTIF(Rules!$B$2:$B$26,M4)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L4)+COUNTIF(Rules!$B$2:$B$29,M4)</f>
         <v>5</v>
       </c>
       <c r="G4" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L4,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M4,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L4,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M4,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H4" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L4,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M4,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L4,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M4,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I4" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L4,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M4,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L4,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M4,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>27</v>
@@ -1576,20 +1621,20 @@
         <v>32</v>
       </c>
       <c r="F5" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L5)+COUNTIF(Rules!$B$2:$B$26,M5)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L5)+COUNTIF(Rules!$B$2:$B$29,M5)</f>
         <v>5</v>
       </c>
       <c r="G5" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L5,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M5,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L5,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M5,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H5" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L5,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M5,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L5,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M5,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I5" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L5,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M5,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L5,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M5,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>33</v>
@@ -1621,20 +1666,20 @@
         <v>26</v>
       </c>
       <c r="F6" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L6)+COUNTIF(Rules!$B$2:$B$26,M6)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L6)+COUNTIF(Rules!$B$2:$B$29,M6)</f>
         <v>5</v>
       </c>
       <c r="G6" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L6,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M6,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L6,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M6,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L6,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M6,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L6,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M6,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L6,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M6,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L6,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M6,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>33</v>
@@ -1666,20 +1711,20 @@
         <v>42</v>
       </c>
       <c r="F7" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L7)+COUNTIF(Rules!$B$2:$B$26,M7)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L7)+COUNTIF(Rules!$B$2:$B$29,M7)</f>
         <v>5</v>
       </c>
       <c r="G7" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L7,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M7,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L7,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M7,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H7" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L7,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M7,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L7,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M7,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I7" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L7,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M7,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L7,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M7,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>33</v>
@@ -1711,20 +1756,20 @@
         <v>42</v>
       </c>
       <c r="F8" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L8)+COUNTIF(Rules!$B$2:$B$26,M8)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L8)+COUNTIF(Rules!$B$2:$B$29,M8)</f>
         <v>5</v>
       </c>
       <c r="G8" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L8,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M8,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L8,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M8,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H8" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L8,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M8,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L8,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M8,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L8,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M8,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L8,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M8,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>33</v>
@@ -1756,20 +1801,20 @@
         <v>32</v>
       </c>
       <c r="F9" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L9)+COUNTIF(Rules!$B$2:$B$26,M9)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L9)+COUNTIF(Rules!$B$2:$B$29,M9)</f>
         <v>5</v>
       </c>
       <c r="G9" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L9,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M9,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L9,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M9,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H9" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L9,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M9,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L9,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M9,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I9" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L9,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M9,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L9,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M9,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>33</v>
@@ -1801,20 +1846,20 @@
         <v>32</v>
       </c>
       <c r="F10" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L10)+COUNTIF(Rules!$B$2:$B$26,M10)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L10)+COUNTIF(Rules!$B$2:$B$29,M10)</f>
         <v>5</v>
       </c>
       <c r="G10" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L10,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M10,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L10,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M10,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H10" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L10,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M10,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L10,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M10,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I10" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L10,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M10,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L10,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M10,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>33</v>
@@ -1846,20 +1891,20 @@
         <v>32</v>
       </c>
       <c r="F11" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L11)+COUNTIF(Rules!$B$2:$B$26,M11)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L11)+COUNTIF(Rules!$B$2:$B$29,M11)</f>
         <v>5</v>
       </c>
       <c r="G11" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L11,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M11,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L11,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M11,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H11" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L11,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M11,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L11,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M11,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I11" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L11,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M11,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L11,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M11,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>0</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>33</v>
@@ -1891,19 +1936,19 @@
         <v>42</v>
       </c>
       <c r="F12" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L12)+COUNTIF(Rules!$B$2:$B$26,M12)</f>
-        <v>4</v>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L12)+COUNTIF(Rules!$B$2:$B$29,M12)</f>
+        <v>5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L12,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M12,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L12,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M12,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H12" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L12,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M12,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L12,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M12,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L12,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M12,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L12,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M12,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>1</v>
       </c>
       <c r="J12" s="2" t="s">
@@ -1936,19 +1981,19 @@
         <v>32</v>
       </c>
       <c r="F13" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L13)+COUNTIF(Rules!$B$2:$B$26,M13)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L13)+COUNTIF(Rules!$B$2:$B$29,M13)</f>
         <v>1</v>
       </c>
       <c r="G13" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L13,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M13,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L13,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M13,Rules!$E$2:$E$29,"In force")</f>
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L13,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M13,Rules!$E$2:$E$26,"Adopted, applies later")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L13,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M13,Rules!$E$2:$E$29,"Adopted, applies later")</f>
         <v>0</v>
       </c>
       <c r="I13" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L13,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M13,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L13,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M13,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>0</v>
       </c>
       <c r="J13" s="2" t="s">
@@ -1981,19 +2026,19 @@
         <v>26</v>
       </c>
       <c r="F14" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L14)+COUNTIF(Rules!$B$2:$B$26,M14)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L14)+COUNTIF(Rules!$B$2:$B$29,M14)</f>
         <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L14,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M14,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L14,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M14,Rules!$E$2:$E$29,"In force")</f>
         <v>2</v>
       </c>
       <c r="H14" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L14,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M14,Rules!$E$2:$E$26,"Adopted, applies later")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L14,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M14,Rules!$E$2:$E$29,"Adopted, applies later")</f>
         <v>0</v>
       </c>
       <c r="I14" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L14,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M14,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L14,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M14,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>0</v>
       </c>
       <c r="J14" s="2" t="s">
@@ -2026,20 +2071,20 @@
         <v>16</v>
       </c>
       <c r="F15" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L15)+COUNTIF(Rules!$B$2:$B$26,M15)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L15)+COUNTIF(Rules!$B$2:$B$29,M15)</f>
+        <v>12</v>
       </c>
       <c r="G15" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L15,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M15,Rules!$E$2:$E$26,"In force")</f>
-        <v>5</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L15,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M15,Rules!$E$2:$E$29,"In force")</f>
+        <v>6</v>
       </c>
       <c r="H15" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L15,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M15,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L15,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M15,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I15" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L15,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M15,Rules!$E$2:$E$26,"Proposal / draft")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L15,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M15,Rules!$E$2:$E$29,"Proposal / draft")</f>
+        <v>4</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>79</v>
@@ -2071,19 +2116,19 @@
         <v>32</v>
       </c>
       <c r="F16" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L16)+COUNTIF(Rules!$B$2:$B$26,M16)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L16)+COUNTIF(Rules!$B$2:$B$29,M16)</f>
+        <v>7</v>
       </c>
       <c r="G16" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L16,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M16,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L16,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M16,Rules!$E$2:$E$29,"In force")</f>
         <v>3</v>
       </c>
       <c r="H16" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L16,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M16,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L16,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M16,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>2</v>
       </c>
       <c r="I16" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L16,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M16,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L16,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M16,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>2</v>
       </c>
       <c r="J16" s="2" t="s">
@@ -2116,19 +2161,19 @@
         <v>32</v>
       </c>
       <c r="F17" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L17)+COUNTIF(Rules!$B$2:$B$26,M17)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L17)+COUNTIF(Rules!$B$2:$B$29,M17)</f>
+        <v>6</v>
       </c>
       <c r="G17" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L17,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M17,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L17,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M17,Rules!$E$2:$E$29,"In force")</f>
         <v>4</v>
       </c>
       <c r="H17" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L17,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M17,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L17,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M17,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>1</v>
       </c>
       <c r="I17" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L17,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M17,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L17,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M17,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>1</v>
       </c>
       <c r="J17" s="2" t="s">
@@ -2161,19 +2206,19 @@
         <v>91</v>
       </c>
       <c r="F18" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L18)+COUNTIF(Rules!$B$2:$B$26,M18)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L18)+COUNTIF(Rules!$B$2:$B$29,M18)</f>
         <v>1</v>
       </c>
       <c r="G18" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L18,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M18,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L18,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M18,Rules!$E$2:$E$29,"In force")</f>
         <v>1</v>
       </c>
       <c r="H18" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L18,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M18,Rules!$E$2:$E$26,"Adopted, applies later")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L18,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M18,Rules!$E$2:$E$29,"Adopted, applies later")</f>
         <v>0</v>
       </c>
       <c r="I18" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L18,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M18,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L18,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M18,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>0</v>
       </c>
       <c r="J18" s="2" t="s">
@@ -2206,19 +2251,19 @@
         <v>42</v>
       </c>
       <c r="F19" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L19)+COUNTIF(Rules!$B$2:$B$26,M19)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L19)+COUNTIF(Rules!$B$2:$B$29,M19)</f>
         <v>0</v>
       </c>
       <c r="G19" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L19,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M19,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L19,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M19,Rules!$E$2:$E$29,"In force")</f>
         <v>0</v>
       </c>
       <c r="H19" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L19,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M19,Rules!$E$2:$E$26,"Adopted, applies later")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L19,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M19,Rules!$E$2:$E$29,"Adopted, applies later")</f>
         <v>0</v>
       </c>
       <c r="I19" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L19,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M19,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L19,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M19,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>0</v>
       </c>
       <c r="J19" s="2" t="s">
@@ -2251,19 +2296,19 @@
         <v>32</v>
       </c>
       <c r="F20" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L20)+COUNTIF(Rules!$B$2:$B$26,M20)</f>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L20)+COUNTIF(Rules!$B$2:$B$29,M20)</f>
         <v>3</v>
       </c>
       <c r="G20" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L20,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M20,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L20,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M20,Rules!$E$2:$E$29,"In force")</f>
         <v>1</v>
       </c>
       <c r="H20" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L20,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M20,Rules!$E$2:$E$26,"Adopted, applies later")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L20,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M20,Rules!$E$2:$E$29,"Adopted, applies later")</f>
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L20,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M20,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L20,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M20,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>1</v>
       </c>
       <c r="J20" s="2" t="s">
@@ -2296,19 +2341,19 @@
         <v>32</v>
       </c>
       <c r="F21" s="4" t="n">
-        <f aca="false">COUNTIF(Rules!$B$2:$B$26,L21)+COUNTIF(Rules!$B$2:$B$26,M21)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(Rules!$B$2:$B$29,L21)+COUNTIF(Rules!$B$2:$B$29,M21)</f>
+        <v>6</v>
       </c>
       <c r="G21" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L21,Rules!$E$2:$E$26,"In force")+COUNTIFS(Rules!$B$2:$B$26,M21,Rules!$E$2:$E$26,"In force")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L21,Rules!$E$2:$E$29,"In force")+COUNTIFS(Rules!$B$2:$B$29,M21,Rules!$E$2:$E$29,"In force")</f>
         <v>4</v>
       </c>
       <c r="H21" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L21,Rules!$E$2:$E$26,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$26,M21,Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L21,Rules!$E$2:$E$29,"Adopted, applies later")+COUNTIFS(Rules!$B$2:$B$29,M21,Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>1</v>
       </c>
       <c r="I21" s="4" t="n">
-        <f aca="false">COUNTIFS(Rules!$B$2:$B$26,L21,Rules!$E$2:$E$26,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$26,M21,Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIFS(Rules!$B$2:$B$29,L21,Rules!$E$2:$E$29,"Proposal / draft")+COUNTIFS(Rules!$B$2:$B$29,M21,Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>1</v>
       </c>
       <c r="J21" s="2" t="s">
@@ -2329,19 +2374,19 @@
         <v>107</v>
       </c>
       <c r="F23" s="5" t="n">
-        <f aca="false">COUNTA(Rules!$A$2:$A$26)</f>
-        <v>25</v>
+        <f aca="false">COUNTA(Rules!$A$2:$A$29)</f>
+        <v>28</v>
       </c>
       <c r="G23" s="5" t="n">
-        <f aca="false">COUNTIF(Rules!$E$2:$E$26,"In force")</f>
-        <v>15</v>
+        <f aca="false">COUNTIF(Rules!$E$2:$E$29,"In force")</f>
+        <v>16</v>
       </c>
       <c r="H23" s="5" t="n">
-        <f aca="false">COUNTIF(Rules!$E$2:$E$26,"Adopted, applies later")</f>
-        <v>4</v>
+        <f aca="false">COUNTIF(Rules!$E$2:$E$29,"Adopted, applies later")</f>
+        <v>6</v>
       </c>
       <c r="I23" s="5" t="n">
-        <f aca="false">COUNTIF(Rules!$E$2:$E$26,"Proposal / draft")</f>
+        <f aca="false">COUNTIF(Rules!$E$2:$E$29,"Proposal / draft")</f>
         <v>6</v>
       </c>
     </row>
@@ -2374,7 +2419,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2548,7 +2593,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -2561,23 +2606,23 @@
       <c r="D6" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="8" t="s">
         <v>147</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2588,7 +2633,7 @@
         <v>62</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>119</v>
@@ -2597,19 +2642,19 @@
         <v>6</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="8" t="s">
         <v>153</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2620,13 +2665,13 @@
         <v>62</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>119</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>90</v>
@@ -2652,7 +2697,7 @@
         <v>62</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>159</v>
@@ -2676,7 +2721,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -2684,16 +2729,16 @@
         <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>166</v>
@@ -2708,15 +2753,15 @@
         <v>169</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>73</v>
+        <v>148</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>170</v>
@@ -2725,19 +2770,19 @@
         <v>6</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="8" t="s">
         <v>174</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2751,57 +2796,57 @@
         <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>119</v>
+        <v>175</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>6</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>180</v>
+        <v>119</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>6</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="I13" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="J13" s="8" t="s">
         <v>184</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2809,13 +2854,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>159</v>
+        <v>185</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>6</v>
@@ -2847,28 +2892,28 @@
         <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E15" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="I15" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -2879,7 +2924,7 @@
         <v>78</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>6</v>
@@ -2900,7 +2945,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -2911,25 +2956,25 @@
         <v>78</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>143</v>
+        <v>202</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>137</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2943,57 +2988,57 @@
         <v>78</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>143</v>
+        <v>170</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>6</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>137</v>
+        <v>175</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>154</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3001,63 +3046,63 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>119</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>90</v>
+        <v>218</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>6</v>
+        <v>175</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>154</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>90</v>
+        <v>223</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3065,83 +3110,83 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>6</v>
+        <v>202</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>137</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>6</v>
+        <v>119</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>154</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>230</v>
+        <v>90</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>143</v>
+        <v>170</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>6</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>236</v>
+        <v>90</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>237</v>
@@ -3156,21 +3201,21 @@
         <v>240</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>137</v>
+        <v>185</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>6</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>241</v>
@@ -3188,18 +3233,18 @@
         <v>245</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>6</v>
@@ -3220,34 +3265,133 @@
         <v>250</v>
       </c>
     </row>
+    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>265</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J26"/>
+  <autoFilter ref="A1:J29"/>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" display="https://eur-lex.europa.eu/eli/reg/2011/1169/oj"/>
     <hyperlink ref="J3" r:id="rId2" display="https://eur-lex.europa.eu/eli/dir/2019/2161/oj"/>
     <hyperlink ref="J4" r:id="rId3" display="https://eur-lex.europa.eu/eli/dir/2024/825/oj"/>
     <hyperlink ref="J5" r:id="rId4" display="https://vinciworks.com/blog/eudr-delayed-again-what-changed-what-is-now-fixed-and-what-businesses-should-do-in-2026/"/>
-    <hyperlink ref="J6" r:id="rId5" display="https://blog.foodsconnected.com/7-key-takeaways-from-the-april-2026-eudr-review"/>
+    <hyperlink ref="J6" r:id="rId5" display="https://eur-lex.europa.eu/eli/reg_del/2026/2102/oj/eng"/>
     <hyperlink ref="J7" r:id="rId6" display="https://eec.eaeunion.org/comission/department/deptexreg/tr/PischevkaMarkirovka.php"/>
     <hyperlink ref="J8" r:id="rId7" display="https://nkprom.ru/news/v-tr-ts-022-2011-pishchevaya-produktsiya-v-chasti-ee-markirovki-i-tr-ts-022-2011-o-bezopasnosti-sred/"/>
     <hyperlink ref="J9" r:id="rId8" display="https://foodsmi.com/zakonodatelstvo/izmeneniya-v-tekhreglamente-na-maslozhirovuyu-produktsiyu/"/>
-    <hyperlink ref="J10" r:id="rId9" display="https://adilet.zan.kz/rus/docs/H13EV000067"/>
-    <hyperlink ref="J11" r:id="rId10" display="https://biz.ligazakon.net/news/231710_prezident-pdpisav-zakon-pro-obmezhennya-vikoristannya-palmovo-ol-u-produktakh-kharchuvannya"/>
-    <hyperlink ref="J12" r:id="rId11" display="https://ngu.com.ua/palmova-oliia-shkoda-sklad-doza-i-etyketka/"/>
-    <hyperlink ref="J13" r:id="rId12" display="https://ansa.gov.md/sites/default/files/documents/Ordine/Ordin%20nr.%20369.pdf"/>
-    <hyperlink ref="J14" r:id="rId13" display="https://www.retail.ru/news/v-rossii-poyavilsya-edinyy-katalog-produktov-bez-palmy-23-dekabrya-2025-272975/"/>
-    <hyperlink ref="J15" r:id="rId14" display="https://www.klerk.ru/buh/articles/713288/"/>
-    <hyperlink ref="J16" r:id="rId15" display="https://www.gazeta.ru/business/2019/07/01/12467725.shtml"/>
-    <hyperlink ref="J17" r:id="rId16" display="https://oleoscope.com/analytics/gosduma-predlozhila-markirovku-dlja-masla/"/>
-    <hyperlink ref="J18" r:id="rId17" display="https://ria.ru/20260722/markirovka-2106133235.html"/>
-    <hyperlink ref="J19" r:id="rId18" display="https://inbusiness.kz/ru/news/v-kazahstane-pochti-vdvoe-rasshirili-markirovku-tovarov"/>
-    <hyperlink ref="J20" r:id="rId19" display="https://kapital.kz/business/134274/maslopererabotchiki-rk-vystupayut-za-ukazaniye-nalichiya-v-produktakh-pal-movogo-masla.html"/>
-    <hyperlink ref="J21" r:id="rId20" display="https://dairynews.today/kz/news/v-kyrgyzstane-obsuzhdayut-ispolzovanie-palmovogo-masla-v-proizvodstve-moloka.html"/>
-    <hyperlink ref="J22" r:id="rId21" display="https://base.spinform.ru/show_doc.fwx?rgn=124770"/>
-    <hyperlink ref="J23" r:id="rId22" display="https://podrobno.uz/cat/obchestvo/v-uzbekistane-vvodyat-obyazatelnyy-laboratornyy-kontrol-palmovogo-masla-i-transzhirov/"/>
-    <hyperlink ref="J24" r:id="rId23" display="https://www.spot.uz/ru/2026/07/30/palm-oil"/>
-    <hyperlink ref="J25" r:id="rId24" display="https://vzglyad.uz/2026/10/09/obsuzhdenie-poryadka-markirovki-rastitelnogo-masla"/>
-    <hyperlink ref="J26" r:id="rId25" display="https://dairynews.today/kz/news/armenia-to-enforce-stricter-labeling-rules-for-dairy-and-meat-products.html"/>
+    <hyperlink ref="J10" r:id="rId9" display="https://base.spinform.ru/show_doc.fwx?rgn=177646"/>
+    <hyperlink ref="J11" r:id="rId10" display="https://adilet.zan.kz/rus/docs/H13EV000067"/>
+    <hyperlink ref="J12" r:id="rId11" display="https://biz.ligazakon.net/news/231710_prezident-pdpisav-zakon-pro-obmezhennya-vikoristannya-palmovo-ol-u-produktakh-kharchuvannya"/>
+    <hyperlink ref="J13" r:id="rId12" display="https://ngu.com.ua/palmova-oliia-shkoda-sklad-doza-i-etyketka/"/>
+    <hyperlink ref="J14" r:id="rId13" display="https://ansa.gov.md/sites/default/files/documents/Ordine/Ordin%20nr.%20369.pdf"/>
+    <hyperlink ref="J15" r:id="rId14" display="https://www.retail.ru/news/v-rossii-poyavilsya-edinyy-katalog-produktov-bez-palmy-23-dekabrya-2025-272975/"/>
+    <hyperlink ref="J16" r:id="rId15" display="https://www.v2b.ru/documents/federalnyy-zakon-ot-02-08-2019-268-fz/"/>
+    <hyperlink ref="J17" r:id="rId16" display="https://www.klerk.ru/buh/articles/713288/"/>
+    <hyperlink ref="J18" r:id="rId17" display="https://www.gazeta.ru/business/2019/07/01/12467725.shtml"/>
+    <hyperlink ref="J19" r:id="rId18" display="https://oleoscope.com/analytics/gosduma-predlozhila-markirovku-dlja-masla/"/>
+    <hyperlink ref="J20" r:id="rId19" display="https://ria.ru/20260722/markirovka-2106133235.html"/>
+    <hyperlink ref="J21" r:id="rId20" display="https://ria.ru/20261024/maslo-2126771171.html"/>
+    <hyperlink ref="J22" r:id="rId21" display="https://inbusiness.kz/ru/news/v-kazahstane-pochti-vdvoe-rasshirili-markirovku-tovarov"/>
+    <hyperlink ref="J23" r:id="rId22" display="https://kapital.kz/business/134274/maslopererabotchiki-rk-vystupayut-za-ukazaniye-nalichiya-v-produktakh-pal-movogo-masla.html"/>
+    <hyperlink ref="J24" r:id="rId23" display="https://dairynews.today/kz/news/v-kyrgyzstane-obsuzhdayut-ispolzovanie-palmovogo-masla-v-proizvodstve-moloka.html"/>
+    <hyperlink ref="J25" r:id="rId24" display="https://base.spinform.ru/show_doc.fwx?rgn=124770"/>
+    <hyperlink ref="J26" r:id="rId25" display="https://podrobno.uz/cat/obchestvo/v-uzbekistane-vvodyat-obyazatelnyy-laboratornyy-kontrol-palmovogo-masla-i-transzhirov/"/>
+    <hyperlink ref="J27" r:id="rId26" display="https://www.spot.uz/ru/2026/07/30/palm-oil"/>
+    <hyperlink ref="J28" r:id="rId27" display="https://vzglyad.uz/2026/10/09/obsuzhdenie-poryadka-markirovki-rastitelnogo-masla"/>
+    <hyperlink ref="J29" r:id="rId28" display="https://dairynews.today/kz/news/armenia-to-enforce-stricter-labeling-rules-for-dairy-and-meat-products.html"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3256,7 +3400,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId26"/>
+  <drawing r:id="rId29"/>
 </worksheet>
 </file>
 
@@ -3274,32 +3418,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="B1" s="12"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3308,7 +3452,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="B6" s="12"/>
     </row>
@@ -3326,7 +3470,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="B9" s="12"/>
     </row>
@@ -3336,7 +3480,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="B11" s="12"/>
     </row>
@@ -3354,31 +3498,31 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="B17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>235</v>
+        <v>196</v>
       </c>
       <c r="B18" s="12"/>
     </row>
@@ -3400,26 +3544,26 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>265</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>